<commit_message>
refresh collectf and meme reporting, roc-pr curvesç
</commit_message>
<xml_diff>
--- a/OUTPUT/direct_A0A0B6P4W3_Yersinia_pestis_CO92.xlsx
+++ b/OUTPUT/direct_A0A0B6P4W3_Yersinia_pestis_CO92.xlsx
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.0242</v>
+        <v>0.02439024390243903</v>
       </c>
     </row>
     <row r="3">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.457</v>
+        <v>0.4570171931227509</v>
       </c>
     </row>
     <row r="4">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.4712</v>
+        <v>0.4712115153938425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>